<commit_message>
docs(requirements): merge 5 extra-feature requirements (F1-F5) into matrix
</commit_message>
<xml_diff>
--- a/需求矩阵-第1组-王浩恩.xlsx
+++ b/需求矩阵-第1组-王浩恩.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BIT-SummerTermProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC253ECD-329F-4092-9320-E0E897A36EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA4FEF1-33EA-4320-B7DF-4B0F65CD5EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3430" yWindow="2280" windowWidth="19200" windowHeight="11710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="需求进度管理表" sheetId="1" r:id="rId1"/>
@@ -109,19 +109,8 @@
     <definedName name="质量保证计划">[4]配置管理计划!$B$206</definedName>
     <definedName name="子活动类型名" comment="#REF!$C$4:$C$36">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -130,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="161">
   <si>
     <t>NO.</t>
   </si>
@@ -162,6 +151,27 @@
     <t>充电用户端</t>
   </si>
   <si>
+    <t>用户信息维护</t>
+  </si>
+  <si>
+    <t>免密注册/登录</t>
+  </si>
+  <si>
+    <t>11 位手机号校验，服务端命中即返回 token 直接登录，未命中自动注册为 用户+后4位 并发 token，提示「注册并登录」。</t>
+  </si>
+  <si>
+    <t>胡晟源</t>
+  </si>
+  <si>
+    <t>×</t>
+  </si>
+  <si>
+    <t>个人信息展示与修改</t>
+  </si>
+  <si>
+    <t>登录后展示默认灰色头像、昵称、钱包余额（元）；改昵称实时落库；展示账户余额；头像上传</t>
+  </si>
+  <si>
     <t>充电站查询</t>
   </si>
   <si>
@@ -171,12 +181,6 @@
     <t>用户可下拉选区域或手动输入地址，程序通过 QNetworkAccessManager 调用腾讯地图 geocoder 接口把地址换算成经纬度；Key 从 config.local.ini 读取、不写死在代码里；解析失败或超时会提示原因并支持重试。</t>
   </si>
   <si>
-    <t>胡晟源</t>
-  </si>
-  <si>
-    <t>×</t>
-  </si>
-  <si>
     <t>附近电站列表展示</t>
   </si>
   <si>
@@ -201,12 +205,6 @@
     <t>△</t>
   </si>
   <si>
-    <t>用户信息维护</t>
-  </si>
-  <si>
-    <t>个人信息展示与修改</t>
-  </si>
-  <si>
     <t>电动汽车充电</t>
   </si>
   <si>
@@ -222,6 +220,9 @@
     <t>完整闭环：charge.reserve 预约空闲桩 → charge.start（校验冻结、余额与桩可用）→ 充电中每 3 秒遥测、服务端按累计电量×站点单价计费 → charge.stop → charge.settle 结算扣款，余额不足转冻结、充值后可续结；历史订单可随时查看。</t>
   </si>
   <si>
+    <t>王浩恩</t>
+  </si>
+  <si>
     <t>PC服务器端</t>
   </si>
   <si>
@@ -291,9 +292,6 @@
     <t>填写站名、地址、经纬度、单价与快慢桩数量即可新增电站（admin.station_create），服务端一并建好对应电桩；新站默认不参与 ML 预测，但照常参与查询、营收与状态统计。</t>
   </si>
   <si>
-    <t>用户管理</t>
-  </si>
-  <si>
     <t>用户列表与查询</t>
   </si>
   <si>
@@ -306,6 +304,24 @@
     <t>在正常与冻结之间切换用户状态（admin.user_set_status）；冻结后该用户不能预约、充值或开始充电，由服务端业务层统一校验；操作全部留痕，冻结与解冻均需弹窗二次确认。</t>
   </si>
   <si>
+    <t>request_log 审计查看器</t>
+  </si>
+  <si>
+    <t>管理端新增「请求日志」页签：按时间倒序分页展示 request_log（requestId、动作、响应码、时间），支持按 requestId 精确查找；实现方式为向后兼容新增一个只读动作 admin.request_log_list（admin token，载荷 {requestId?,limit?,offset?}），不进入冒烟调用清单；开工前须经 #2 确认兼容性并同步 interface-contract.md。</t>
+  </si>
+  <si>
+    <t>庞项祯</t>
+  </si>
+  <si>
+    <t>系统健康</t>
+  </si>
+  <si>
+    <t>健康自检面板</t>
+  </si>
+  <si>
+    <t>管理端新增「系统健康」页签：一屏自检清单——服务状态（system.health）、快照版本一致性（health.snapshotVersion 与 DB snapshot_meta 比对）、活动预测批次与新鲜度（activatedAt 距今）、模拟器连接状态，每项绿勾/红叉；答辩开场/收尾展示「自检全绿」，现场异常时为第一排障入口。</t>
+  </si>
+  <si>
     <t>数据库端</t>
   </si>
   <si>
@@ -345,52 +361,19 @@
     <t>9月2日</t>
   </si>
   <si>
-    <t>大数据可视化大屏</t>
-  </si>
-  <si>
-    <t>数据展示</t>
-  </si>
-  <si>
-    <t>业务健康度看板</t>
-  </si>
-  <si>
-    <t>单页 ECharts 5.6.0 大屏，所有资源本地化、零外部依赖、不登录不写数据；页面包含 4 张 KPI 卡（今日营收/充电量/订单/在线率）、近 7 日营收柱状图、24 小时实际与预测负荷双曲线（含高峰标记与站点选择器）、桩状态环形图、站点利用率排行、经纬度散点与实时事件流。</t>
-  </si>
-  <si>
-    <t>王浩恩</t>
-  </si>
-  <si>
-    <t>数据接入</t>
-  </si>
-  <si>
-    <t>快照轮询与降级</t>
-  </si>
-  <si>
-    <t>唯一数据源是服务端原子生成的 JSON 快照，每 2 秒同源轮询并绕过缓存；渲染前用 validateSnapshot 做 v1 全量校验（19 项规则），校验失败的数据不上屏；超过 10 秒未成功获取即标记 stale 并保留旧数据，另有 cached/error 两种降级态与本地兜底快照，断网或数据异常时不白屏。</t>
-  </si>
-  <si>
-    <t>9月6日</t>
-  </si>
-  <si>
-    <t>机器学习智能分析</t>
-  </si>
-  <si>
-    <t>充电负荷预测</t>
-  </si>
-  <si>
-    <t>负荷智能预测</t>
-  </si>
-  <si>
-    <t>读取 12,960 行历史数据，按时间顺序切分 62 天训练/14 天验证/14 天测试（不随机打乱，防止数据泄露）；以「昨日同一时刻」为 seasonal-naive 基线，与 Ridge 回归按验证集择优选用；按 1h/6h/24h 汇报 MAE/WAPE；输出 6 站×24 小时=144 条预测，并对负荷、占用、空闲做物理范围约束。</t>
-  </si>
-  <si>
-    <t>庞项祯</t>
-  </si>
-  <si>
-    <t>智能推荐与预警</t>
-  </si>
-  <si>
-    <t>ML 通过与服务端相同的 v1 TCP 协议把 144 条预测一次性提交（forecast.publish），服务端单事务校验后入库，发布失败保留上一份可用结果不覆盖；用户端据此展示未来 1 小时预计空闲桩数与拥堵等级（&lt;50% 低、&lt;80% 中、≥80% 高），优先推荐低拥堵站点；占用率≥80% 的站触发负荷预警并标出高峰时段。</t>
+    <t>演示导演模式</t>
+  </si>
+  <si>
+    <t>模拟器新增一键剧本时间轴：自动执行「正常运行 30s → 注入 2 个故障 → 等待/提示远程重启 → 恢复 → 高峰模式」，每步在事件日志同步解说文字；可选时间压缩档位（模拟时钟与墙钟解耦，如 1 秒 = 10 分钟）用于演示 24 小时负荷形态；安全约束：加速仅作用于遥测推进速率与模拟时间戳（recordedAt 由模拟器上报），存在活动订单时自动回落正常速率；复用 TelemetryEngine 与 telemetry.push/simulator.fault_set 既有协议，零协议、零数据库改动。</t>
+  </si>
+  <si>
+    <t>数据质量保障</t>
+  </si>
+  <si>
+    <t>数据库一致性体检</t>
+  </si>
+  <si>
+    <t>Python 命令行工具对 SQLite 数据库一键体检，输出终端 PASS/FAIL 报告与 JSON 工件（runtime/reports/）：第一层数据库健康（PRAGMA integrity_check、外键检查、唯一约束验证）；第二层业务不变量（订单金额=电量×站点单价整数分零误差、同一用户最多一个活动订单、每个 charging 桩恰对应一张 charging 订单、活动预测批次恰 144 条且无负值/越界、snapshot_meta 版本单调递增、用户余额非负、状态字段均为合法枚举）；每轮彩排后运行一次并归档证据链。</t>
   </si>
   <si>
     <t>需求进度管理表</t>
@@ -571,19 +554,91 @@
     <t>未开始，今天完成，下周一验收</t>
   </si>
   <si>
-    <t>免密注册/登录</t>
-  </si>
-  <si>
-    <t>11 位手机号校验，服务端命中即返回 token 直接登录，未命中自动注册为 用户+后4位 并发 token，提示「注册并登录」。</t>
-  </si>
-  <si>
-    <t>登录后展示默认灰色头像、昵称、钱包余额（元）；改昵称实时落库；展示账户余额；头像上传</t>
+    <t>充电过程页</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>审计</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="MS PGothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>日志</t>
+    </r>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>用户管理</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>站点信息</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>实时计费和预警</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>在充电页三层做厚「当前订单页」：基础层显示所在站点、桩编号与快/慢充类型；</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>扩展层轮询 order.current 展示累计电量与服务端实时计费金额，并用相邻两次电量差÷间隔自算功率绘制曲线（零协议变更）；预警层在「余额-已计费金额」低于阈值时本地弹窗提醒，余额耗尽由服务端按既有规则强制停止计费（INSUFFICIENT_BALANCE），页面明示「余额不足已停止计费，充值后完成结算」；结算后订单详情展示文本电子小票，标注「模拟结算凭证，非支付凭证」。</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>数据存储</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>SQLite 数据库 v1 共 13 张业务表，带外键、CHECK 与部分唯一索引等约束；固定种子 seed=20260901 生成 6 站、48 桩、30 用户、30 天订单与 90 天共 12,960 条历史数据，同一种子生成结果哈希完全一致；开启 WAL 与外键，写库超时 3 秒，金额一律按整数分存储。</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>数据处理</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>通信与数据构建</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>通信采用 4 字节长度头 + JSON 的 TCP 帧协议（上限 1MiB），正确处理粘包与半包，非法数据立即断开；权限分 admin/user/simulator/ml 四种角色共 27 个动作、统一 17 个错误码，request_log 留痕；数据侧用固定种子构建并封版 demo.db，导出 12,960 行历史给 ML、回灌 144 条预测后生成 manifest 与 SHA-256，结果可复现。</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>△</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>数据仿真</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>Qt 桌面小程序模拟真实充电桩：TelemetryEngine 按固定节奏每 3 秒上报一次电量遥测，可手动注入或解除故障；走与服务端相同的 v1 TCP 帧协议，断线自动重连并用有界队列缓存；纯内存状态机，不写数据库、不上报金额；附带 3 组 ctest 与一次无界面冒烟验证。</t>
+    <phoneticPr fontId="28" type="noConversion"/>
+  </si>
+  <si>
+    <t>数据库端</t>
+    <phoneticPr fontId="19" type="noConversion"/>
   </si>
   <si>
     <r>
       <rPr>
         <b/>
-        <sz val="26"/>
+        <sz val="22"/>
         <rFont val="宋体"/>
         <family val="3"/>
         <charset val="134"/>
@@ -615,7 +670,7 @@
         <b/>
         <sz val="9"/>
         <rFont val="Segoe UI Symbol"/>
-        <family val="2"/>
+        <family val="3"/>
       </rPr>
       <t>✓</t>
     </r>
@@ -629,7 +684,7 @@
       </rPr>
       <t>：已完成</t>
     </r>
-    <phoneticPr fontId="20" type="noConversion"/>
+    <phoneticPr fontId="19" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -637,13 +692,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="178" formatCode="mmm"/>
-    <numFmt numFmtId="179" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="180" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="_(&quot;\&quot;* #,##0_);_(&quot;\&quot;* \(#,##0\);_(&quot;\&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="182" formatCode="_(&quot;\&quot;* #,##0_);_(&quot;\&quot;* \(#,##0\);_(&quot;\&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="mmm"/>
+    <numFmt numFmtId="177" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_(&quot;\&quot;* #,##0_);_(&quot;\&quot;* \(#,##0\);_(&quot;\&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="179" formatCode="_(&quot;\&quot;* #,##0_);_(&quot;\&quot;* \(#,##0\);_(&quot;\&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -674,12 +729,6 @@
       <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -782,6 +831,43 @@
     </font>
     <font>
       <b/>
+      <sz val="14"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="MS PGothic"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <name val="宋体"/>
       <family val="3"/>
@@ -791,18 +877,11 @@
       <b/>
       <sz val="9"/>
       <name val="Segoe UI Symbol"/>
-      <family val="2"/>
+      <family val="3"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="26"/>
+      <sz val="22"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -822,7 +901,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -1024,48 +1103,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="15" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="15" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="177" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="18" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="179" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="180" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="181" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="19" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="178" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+  <cellXfs count="66">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
@@ -1132,103 +1220,148 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="20" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="20" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="27" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="10" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="11" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="15" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="27" fillId="0" borderId="11" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="10" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="11" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="4" fillId="0" borderId="12" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="58" fontId="4" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="4" fillId="0" borderId="10" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="4" fillId="0" borderId="11" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="4" fillId="0" borderId="12" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="21" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="21" fillId="0" borderId="3" xfId="12" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="12" applyFont="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="23">
-    <cellStyle name="Calc Currency (0)" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="ColLevel_1" xfId="2" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="Date" xfId="3" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="Header1" xfId="4" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="Header2" xfId="5" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="New Times Roman" xfId="6" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
-    <cellStyle name="Normal_#10-Headcount" xfId="7" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
-    <cellStyle name="RowLevel_1" xfId="8" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="標準_(D)日程計画" xfId="9" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="表示済みのハイパーリンク_02_1st_2ndOTP対応機能一覧_一応完成版" xfId="10" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="Calc Currency (0)" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="ColLevel_1" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Date" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Header1" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Header2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="New Times Roman" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal_#10-Headcount" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="RowLevel_1" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="標準_(D)日程計画" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="表示済みのハイパーリンク_02_1st_2ndOTP対応機能一覧_一応完成版" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规_需求跟踪矩阵" xfId="11" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="超级链接_IPPR-B" xfId="12" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
-    <cellStyle name="段落标题1" xfId="13" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
-    <cellStyle name="段落标题2" xfId="14" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
-    <cellStyle name="桁区切り [0.00]_(D)日程計画" xfId="15" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
-    <cellStyle name="桁区切り_(D)日程計画" xfId="16" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
-    <cellStyle name="普通_laroux" xfId="17" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
-    <cellStyle name="千位[0]_laroux" xfId="18" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
-    <cellStyle name="千位_laroux" xfId="19" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
-    <cellStyle name="通貨 [0.00]_(D)日程計画" xfId="20" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
-    <cellStyle name="通貨_(D)日程計画" xfId="21" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
-    <cellStyle name="样式 1" xfId="22" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
+    <cellStyle name="常规_需求跟踪矩阵" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="超级链接_IPPR-B" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="段落标题1" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="段落标题2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="桁区切り [0.00]_(D)日程計画" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="桁区切り_(D)日程計画" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="普通_laroux" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="千位[0]_laroux" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="千位_laroux" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="通貨 [0.00]_(D)日程計画" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="通貨_(D)日程計画" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="样式 1" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1691,7 +1824,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z168"/>
+  <dimension ref="A1:Z169"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.6328125" style="1" customWidth="1"/>
@@ -1699,7 +1832,7 @@
     <col min="3" max="3" width="20.1796875" style="2" customWidth="1"/>
     <col min="4" max="4" width="17.6328125" style="2" customWidth="1"/>
     <col min="5" max="5" width="22.6328125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="62.6328125" style="47" customWidth="1"/>
+    <col min="6" max="6" width="62.6328125" style="38" customWidth="1"/>
     <col min="7" max="7" width="9.6328125" style="1" customWidth="1"/>
     <col min="8" max="8" width="11.6328125" style="3" customWidth="1"/>
     <col min="9" max="9" width="7.1796875" style="3" customWidth="1"/>
@@ -1708,30 +1841,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="41.25" customHeight="1">
-      <c r="A1" s="48" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
+      <c r="A1" s="58" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="63"/>
     </row>
     <row r="2" spans="1:10" ht="21" customHeight="1">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
+      <c r="A2" s="61"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" s="1" customFormat="1" ht="24" customHeight="1">
       <c r="B3" s="25" t="s">
@@ -1746,7 +1879,7 @@
       <c r="E3" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="46" t="s">
+      <c r="F3" s="37" t="s">
         <v>4</v>
       </c>
       <c r="G3" s="26" t="s">
@@ -1766,677 +1899,813 @@
       <c r="B4" s="28">
         <v>1</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>146</v>
-      </c>
-      <c r="F4" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="G4" s="39" t="s">
+      <c r="D4" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="41">
+      <c r="H4" s="34">
         <v>46267</v>
       </c>
-      <c r="I4" s="41" t="s">
+      <c r="I4" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="39"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B5" s="28">
         <v>2</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="G5" s="39" t="s">
+      <c r="C5" s="54"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="41">
+      <c r="H5" s="34">
         <v>46270</v>
       </c>
-      <c r="I5" s="41" t="s">
+      <c r="I5" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="39"/>
+      <c r="J5" s="32"/>
     </row>
     <row r="6" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B6" s="28">
         <v>3</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="38" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="39" t="s">
+      <c r="C6" s="54"/>
+      <c r="D6" s="51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="41">
+      <c r="H6" s="34">
         <v>46269</v>
       </c>
-      <c r="I6" s="41" t="s">
+      <c r="I6" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="44"/>
+      <c r="J6" s="36"/>
     </row>
     <row r="7" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B7" s="28">
         <v>4</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="39" t="s">
+      <c r="C7" s="54"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="32" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="41">
+      <c r="H7" s="34">
         <v>46269</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="39"/>
+      <c r="J7" s="32"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B8" s="28">
         <v>5</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="40" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="39" t="s">
+      <c r="C8" s="54"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="41">
+      <c r="H8" s="34">
         <v>46269</v>
       </c>
-      <c r="I8" s="41" t="s">
+      <c r="I8" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="39"/>
+      <c r="J8" s="32"/>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B9" s="28">
         <v>6</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="39" t="s">
+      <c r="C9" s="54"/>
+      <c r="D9" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="41">
+      <c r="H9" s="34">
         <v>46270</v>
       </c>
-      <c r="I9" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="39"/>
+      <c r="I9" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="32"/>
     </row>
     <row r="10" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B10" s="28">
         <v>7</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="39" t="s">
+      <c r="C10" s="54"/>
+      <c r="D10" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="41">
+      <c r="H10" s="34">
         <v>46268</v>
       </c>
-      <c r="I10" s="41" t="s">
+      <c r="I10" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="39"/>
+      <c r="J10" s="32"/>
     </row>
     <row r="11" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B11" s="28">
         <v>8</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="39" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="40" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="39" t="s">
+      <c r="C11" s="54"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="34">
         <v>46268</v>
       </c>
-      <c r="I11" s="41" t="s">
+      <c r="I11" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="39"/>
+      <c r="J11" s="32"/>
     </row>
     <row r="12" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
-      <c r="B12" s="28">
-        <v>9</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="40" t="s">
+      <c r="B12" s="28"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="56" t="s">
+        <v>144</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F12" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="G12" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H12" s="30">
-        <v>46267</v>
-      </c>
-      <c r="I12" s="30" t="s">
+      <c r="H12" s="34">
+        <v>46273</v>
+      </c>
+      <c r="I12" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="28"/>
+      <c r="J12" s="32"/>
     </row>
     <row r="13" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
-      <c r="B13" s="28">
-        <v>10</v>
-      </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H13" s="30">
-        <v>46270</v>
-      </c>
-      <c r="I13" s="30" t="s">
+      <c r="B13" s="28"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="34">
+        <v>46274</v>
+      </c>
+      <c r="I13" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="28"/>
+      <c r="J13" s="32"/>
     </row>
     <row r="14" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B14" s="28">
-        <v>11</v>
-      </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="36"/>
+        <v>9</v>
+      </c>
+      <c r="C14" s="64" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>35</v>
+      </c>
       <c r="E14" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H14" s="30">
-        <v>46270</v>
-      </c>
-      <c r="I14" s="30" t="s">
+      <c r="H14" s="29">
+        <v>46267</v>
+      </c>
+      <c r="I14" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J14" s="28"/>
     </row>
     <row r="15" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B15" s="28">
-        <v>12</v>
-      </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="52"/>
+      <c r="D15" s="49" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="28" t="s">
+      <c r="F15" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="40" t="s">
-        <v>42</v>
-      </c>
       <c r="G15" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H15" s="30">
+        <v>38</v>
+      </c>
+      <c r="H15" s="29">
         <v>46270</v>
       </c>
-      <c r="I15" s="30" t="s">
+      <c r="I15" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J15" s="28"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B16" s="28">
-        <v>13</v>
-      </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="52"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="F16" s="40" t="s">
-        <v>45</v>
-      </c>
       <c r="G16" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H16" s="30">
+        <v>38</v>
+      </c>
+      <c r="H16" s="29">
         <v>46270</v>
       </c>
-      <c r="I16" s="30" t="s">
+      <c r="I16" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J16" s="28"/>
     </row>
     <row r="17" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B17" s="28">
-        <v>14</v>
-      </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="36"/>
+        <v>12</v>
+      </c>
+      <c r="C17" s="52"/>
+      <c r="D17" s="28" t="s">
+        <v>44</v>
+      </c>
       <c r="E17" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="F17" s="40" t="s">
-        <v>47</v>
-      </c>
       <c r="G17" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H17" s="30">
+        <v>38</v>
+      </c>
+      <c r="H17" s="29">
         <v>46270</v>
       </c>
-      <c r="I17" s="30" t="s">
+      <c r="I17" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J17" s="28"/>
     </row>
     <row r="18" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B18" s="28">
-        <v>15</v>
-      </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="52"/>
+      <c r="D18" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="F18" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="F18" s="40" t="s">
-        <v>50</v>
-      </c>
       <c r="G18" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H18" s="30">
+        <v>38</v>
+      </c>
+      <c r="H18" s="29">
         <v>46270</v>
       </c>
-      <c r="I18" s="30" t="s">
+      <c r="I18" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J18" s="28"/>
     </row>
     <row r="19" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B19" s="28">
-        <v>16</v>
-      </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="36"/>
+        <v>14</v>
+      </c>
+      <c r="C19" s="52"/>
+      <c r="D19" s="50"/>
       <c r="E19" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="40" t="s">
-        <v>52</v>
-      </c>
       <c r="G19" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H19" s="30">
+        <v>38</v>
+      </c>
+      <c r="H19" s="29">
         <v>46270</v>
       </c>
-      <c r="I19" s="30" t="s">
+      <c r="I19" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J19" s="28"/>
     </row>
     <row r="20" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B20" s="28">
-        <v>17</v>
-      </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="52"/>
+      <c r="D20" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="F20" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="F20" s="40" t="s">
-        <v>55</v>
-      </c>
       <c r="G20" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H20" s="30">
+        <v>38</v>
+      </c>
+      <c r="H20" s="29">
         <v>46270</v>
       </c>
-      <c r="I20" s="30" t="s">
+      <c r="I20" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J20" s="28"/>
     </row>
     <row r="21" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B21" s="28">
-        <v>18</v>
-      </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="36"/>
+        <v>16</v>
+      </c>
+      <c r="C21" s="52"/>
+      <c r="D21" s="50"/>
       <c r="E21" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="F21" s="40" t="s">
-        <v>57</v>
-      </c>
       <c r="G21" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="H21" s="30">
+        <v>38</v>
+      </c>
+      <c r="H21" s="29">
         <v>46270</v>
       </c>
-      <c r="I21" s="30" t="s">
+      <c r="I21" s="29" t="s">
         <v>14</v>
       </c>
       <c r="J21" s="28"/>
     </row>
     <row r="22" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B22" s="28">
-        <v>19</v>
-      </c>
-      <c r="C22" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="52"/>
+      <c r="D22" s="65" t="s">
+        <v>146</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="F22" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="E22" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" s="40" t="s">
-        <v>61</v>
-      </c>
       <c r="G22" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="H22" s="30">
-        <v>46267</v>
-      </c>
-      <c r="I22" s="31" t="s">
-        <v>63</v>
+        <v>38</v>
+      </c>
+      <c r="H22" s="29">
+        <v>46270</v>
+      </c>
+      <c r="I22" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="J22" s="28"/>
     </row>
     <row r="23" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B23" s="28">
-        <v>20</v>
-      </c>
-      <c r="C23" s="33"/>
-      <c r="D23" s="29" t="s">
-        <v>64</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C23" s="52"/>
+      <c r="D23" s="50"/>
       <c r="E23" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F23" s="40" t="s">
-        <v>66</v>
+        <v>59</v>
+      </c>
+      <c r="F23" s="33" t="s">
+        <v>60</v>
       </c>
       <c r="G23" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="H23" s="30">
-        <v>46268</v>
-      </c>
-      <c r="I23" s="31" t="s">
-        <v>22</v>
+        <v>38</v>
+      </c>
+      <c r="H23" s="29">
+        <v>46270</v>
+      </c>
+      <c r="I23" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="J23" s="28"/>
     </row>
     <row r="24" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B24" s="28">
-        <v>21</v>
-      </c>
-      <c r="C24" s="34"/>
-      <c r="D24" s="28" t="s">
-        <v>67</v>
+        <v>27</v>
+      </c>
+      <c r="C24" s="52"/>
+      <c r="D24" s="39" t="s">
+        <v>145</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" s="40" t="s">
-        <v>69</v>
+        <v>61</v>
+      </c>
+      <c r="F24" s="33" t="s">
+        <v>62</v>
       </c>
       <c r="G24" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="H24" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="I24" s="31" t="s">
-        <v>22</v>
+        <v>63</v>
+      </c>
+      <c r="H24" s="29">
+        <v>46271</v>
+      </c>
+      <c r="I24" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="J24" s="28"/>
     </row>
-    <row r="25" spans="2:10" s="1" customFormat="1" ht="86" hidden="1" customHeight="1">
+    <row r="25" spans="2:10" s="1" customFormat="1" ht="86" customHeight="1">
       <c r="B25" s="28">
-        <v>22</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>71</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>72</v>
+        <v>28</v>
+      </c>
+      <c r="C25" s="50"/>
+      <c r="D25" s="40" t="s">
+        <v>64</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="40" t="s">
-        <v>74</v>
+        <v>65</v>
+      </c>
+      <c r="F25" s="33" t="s">
+        <v>66</v>
       </c>
       <c r="G25" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="H25" s="30">
-        <v>46271</v>
-      </c>
-      <c r="I25" s="30" t="s">
-        <v>22</v>
+        <v>63</v>
+      </c>
+      <c r="H25" s="29">
+        <v>46272</v>
+      </c>
+      <c r="I25" s="29" t="s">
+        <v>14</v>
       </c>
       <c r="J25" s="28"/>
     </row>
     <row r="26" spans="2:10" s="1" customFormat="1" ht="86" hidden="1" customHeight="1">
       <c r="B26" s="28">
-        <v>23</v>
-      </c>
-      <c r="C26" s="34"/>
-      <c r="D26" s="29" t="s">
-        <v>76</v>
+        <v>19</v>
+      </c>
+      <c r="C26" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>68</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="F26" s="40" t="s">
-        <v>78</v>
+        <v>69</v>
+      </c>
+      <c r="F26" s="33" t="s">
+        <v>70</v>
       </c>
       <c r="G26" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="H26" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="I26" s="31" t="s">
-        <v>22</v>
+        <v>71</v>
+      </c>
+      <c r="H26" s="29">
+        <v>46267</v>
+      </c>
+      <c r="I26" s="30" t="s">
+        <v>72</v>
       </c>
       <c r="J26" s="28"/>
     </row>
     <row r="27" spans="2:10" s="1" customFormat="1" ht="86" hidden="1" customHeight="1">
       <c r="B27" s="28">
-        <v>24</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="D27" s="35" t="s">
-        <v>81</v>
+        <v>20</v>
+      </c>
+      <c r="C27" s="46"/>
+      <c r="D27" s="31" t="s">
+        <v>73</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="F27" s="40" t="s">
-        <v>83</v>
+        <v>74</v>
+      </c>
+      <c r="F27" s="33" t="s">
+        <v>75</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="H27" s="30">
-        <v>46270</v>
+        <v>71</v>
+      </c>
+      <c r="H27" s="29">
+        <v>46268</v>
       </c>
       <c r="I27" s="30" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="J27" s="28"/>
     </row>
     <row r="28" spans="2:10" s="1" customFormat="1" ht="86" hidden="1" customHeight="1">
       <c r="B28" s="28">
+        <v>21</v>
+      </c>
+      <c r="C28" s="46"/>
+      <c r="D28" s="49" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="G28" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="H28" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="I28" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" s="28"/>
+    </row>
+    <row r="29" spans="2:10" s="1" customFormat="1" ht="86" hidden="1" customHeight="1">
+      <c r="B29" s="28">
+        <v>29</v>
+      </c>
+      <c r="C29" s="46"/>
+      <c r="D29" s="50"/>
+      <c r="E29" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="F29" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="G29" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="H29" s="28">
+        <v>46271</v>
+      </c>
+      <c r="I29" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="28"/>
+    </row>
+    <row r="30" spans="2:10" ht="86" customHeight="1">
+      <c r="B30" s="28">
+        <v>30</v>
+      </c>
+      <c r="C30" s="48" t="s">
+        <v>159</v>
+      </c>
+      <c r="D30" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="F30" s="42" t="s">
+        <v>152</v>
+      </c>
+      <c r="G30" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="H30" s="42">
+        <v>46267</v>
+      </c>
+      <c r="I30" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="J30" s="28"/>
+    </row>
+    <row r="31" spans="2:10" ht="84.5" customHeight="1">
+      <c r="B31" s="28">
+        <v>22</v>
+      </c>
+      <c r="C31" s="48"/>
+      <c r="D31" s="44" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="41" t="s">
+        <v>154</v>
+      </c>
+      <c r="F31" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="G31" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="H31" s="42">
+        <v>46268</v>
+      </c>
+      <c r="I31" s="43" t="s">
+        <v>156</v>
+      </c>
+      <c r="J31" s="28"/>
+    </row>
+    <row r="32" spans="2:10" ht="86" customHeight="1">
+      <c r="B32" s="28">
+        <v>23</v>
+      </c>
+      <c r="C32" s="48"/>
+      <c r="D32" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="F32" s="42" t="s">
+        <v>158</v>
+      </c>
+      <c r="G32" s="41" t="s">
+        <v>71</v>
+      </c>
+      <c r="H32" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="I32" s="43" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="28"/>
+    </row>
+    <row r="33" spans="2:10" ht="86" customHeight="1">
+      <c r="B33" s="28">
+        <v>24</v>
+      </c>
+      <c r="C33" s="48"/>
+      <c r="D33" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="E33" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="F33" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="G33" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="H33" s="29">
+        <v>46271</v>
+      </c>
+      <c r="I33" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="J33" s="28"/>
+    </row>
+    <row r="34" spans="2:10" ht="86" hidden="1" customHeight="1">
+      <c r="B34" s="28">
         <v>25</v>
       </c>
-      <c r="C28" s="34"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="F28" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="G28" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="H28" s="30">
-        <v>46270</v>
-      </c>
-      <c r="I28" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="J28" s="28"/>
-    </row>
-    <row r="29" spans="2:10" ht="86" customHeight="1">
-      <c r="B29" s="23"/>
-    </row>
-    <row r="30" spans="2:10" ht="86" customHeight="1">
-      <c r="B30" s="23"/>
-    </row>
-    <row r="31" spans="2:10">
-      <c r="B31" s="23"/>
-    </row>
-    <row r="32" spans="2:10">
-      <c r="B32" s="23"/>
-    </row>
-    <row r="33" spans="2:2">
-      <c r="B33" s="23"/>
-    </row>
-    <row r="34" spans="2:2">
-      <c r="B34" s="23"/>
-    </row>
-    <row r="35" spans="2:2">
+      <c r="C34" s="47"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="33"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="28"/>
+    </row>
+    <row r="35" spans="2:10" ht="14" hidden="1">
       <c r="B35" s="23"/>
-    </row>
-    <row r="36" spans="2:2">
+      <c r="C35" s="47"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="42"/>
+      <c r="G35" s="41"/>
+      <c r="H35" s="42"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="41"/>
+    </row>
+    <row r="36" spans="2:10" ht="14" hidden="1">
       <c r="B36" s="23"/>
-    </row>
-    <row r="37" spans="2:2">
+      <c r="C36" s="47"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="41"/>
+      <c r="H36" s="42"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="41"/>
+    </row>
+    <row r="37" spans="2:10" ht="14" hidden="1">
       <c r="B37" s="23"/>
-    </row>
-    <row r="38" spans="2:2">
+      <c r="C37" s="47"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="41"/>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="41"/>
+    </row>
+    <row r="38" spans="2:10" hidden="1">
       <c r="B38" s="23"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:10">
       <c r="B39" s="23"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:10">
       <c r="B40" s="23"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:10">
       <c r="B41" s="23"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:10">
       <c r="B42" s="23"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:10">
       <c r="B43" s="23"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:10">
       <c r="B44" s="23"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:10">
       <c r="B45" s="23"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:10">
       <c r="B46" s="23"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:10">
       <c r="B47" s="23"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:10">
       <c r="B48" s="23"/>
     </row>
     <row r="49" spans="2:2">
@@ -2799,24 +3068,26 @@
     <row r="168" spans="2:2">
       <c r="B168" s="23"/>
     </row>
+    <row r="169" spans="2:2">
+      <c r="B169" s="23"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="C14:C25"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D22:D23"/>
     <mergeCell ref="D18:D19"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="C4:C13"/>
+    <mergeCell ref="D12:D13"/>
     <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="C4:C11"/>
-    <mergeCell ref="C12:C21"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="C27:C28"/>
   </mergeCells>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="0.98" bottom="0.98" header="0.51" footer="0.51"/>
   <pageSetup paperSize="9" scale="14" orientation="landscape"/>
@@ -2846,7 +3117,7 @@
   <sheetData>
     <row r="1" spans="2:12" ht="41.25" customHeight="1">
       <c r="B1" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -2855,7 +3126,7 @@
     </row>
     <row r="2" spans="2:12" ht="21" customHeight="1">
       <c r="B2" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -2891,10 +3162,10 @@
         <v>8</v>
       </c>
       <c r="K3" s="11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="2:12" s="1" customFormat="1" ht="34" customHeight="1">
@@ -2902,30 +3173,30 @@
         <v>1</v>
       </c>
       <c r="C4" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="F4" s="13" t="s">
         <v>92</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>94</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="15">
         <v>43339</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J4" s="17"/>
       <c r="K4" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L4" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -2935,24 +3206,24 @@
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
       <c r="E5" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="15">
         <v>43339</v>
       </c>
       <c r="I5" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J5" s="17"/>
       <c r="K5" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L5" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="2:12" s="1" customFormat="1" ht="39" customHeight="1">
@@ -2960,30 +3231,30 @@
         <v>3</v>
       </c>
       <c r="C6" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="F6" s="19" t="s">
         <v>100</v>
-      </c>
-      <c r="E6" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" s="19" t="s">
-        <v>102</v>
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="15">
         <v>43340</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J6" s="17"/>
       <c r="K6" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -2993,24 +3264,24 @@
       <c r="C7" s="19"/>
       <c r="D7" s="19"/>
       <c r="E7" s="19" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G7" s="14"/>
       <c r="H7" s="15">
         <v>43340</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J7" s="17"/>
       <c r="K7" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L7" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3020,7 +3291,7 @@
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
       <c r="E8" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F8" s="19"/>
       <c r="G8" s="14"/>
@@ -3028,14 +3299,14 @@
         <v>43339</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J8" s="17"/>
       <c r="K8" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L8" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3044,27 +3315,27 @@
       </c>
       <c r="C9" s="19"/>
       <c r="D9" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="19" t="s">
         <v>106</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>108</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="15">
         <v>43339</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J9" s="17"/>
       <c r="K9" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L9" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3074,24 +3345,24 @@
       <c r="C10" s="19"/>
       <c r="D10" s="19"/>
       <c r="E10" s="19" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="15">
         <v>43340</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J10" s="17"/>
       <c r="K10" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L10" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3101,24 +3372,24 @@
       <c r="C11" s="19"/>
       <c r="D11" s="19"/>
       <c r="E11" s="19" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G11" s="14"/>
       <c r="H11" s="15">
         <v>43340</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J11" s="17"/>
       <c r="K11" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L11" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3128,24 +3399,24 @@
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
       <c r="E12" s="19" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="15">
         <v>43341</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J12" s="17"/>
       <c r="K12" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L12" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3154,27 +3425,27 @@
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="F13" s="19" t="s">
         <v>115</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>117</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="15">
         <v>43339</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J13" s="17"/>
       <c r="K13" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L13" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3184,24 +3455,24 @@
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
       <c r="E14" s="19" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G14" s="14"/>
       <c r="H14" s="15">
         <v>43339</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J14" s="17"/>
       <c r="K14" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3211,7 +3482,7 @@
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
       <c r="E15" s="19" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="14"/>
@@ -3219,14 +3490,14 @@
         <v>43340</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J15" s="17"/>
       <c r="K15" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L15" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3236,7 +3507,7 @@
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
       <c r="E16" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F16" s="19"/>
       <c r="G16" s="14"/>
@@ -3244,14 +3515,14 @@
         <v>43340</v>
       </c>
       <c r="I16" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J16" s="17"/>
       <c r="K16" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3261,7 +3532,7 @@
       <c r="C17" s="19"/>
       <c r="D17" s="19"/>
       <c r="E17" s="19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F17" s="19"/>
       <c r="G17" s="14"/>
@@ -3269,14 +3540,14 @@
         <v>43339</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J17" s="17"/>
       <c r="K17" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L17" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3284,30 +3555,30 @@
         <v>15</v>
       </c>
       <c r="C18" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>122</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>124</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="15">
         <v>43340</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J18" s="17"/>
       <c r="K18" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L18" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3317,24 +3588,24 @@
       <c r="C19" s="19"/>
       <c r="D19" s="19"/>
       <c r="E19" s="19" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="15">
         <v>43340</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J19" s="17"/>
       <c r="K19" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L19" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3344,7 +3615,7 @@
       <c r="C20" s="19"/>
       <c r="D20" s="19"/>
       <c r="E20" s="19" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F20" s="19"/>
       <c r="G20" s="14"/>
@@ -3352,14 +3623,14 @@
         <v>43342</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J20" s="17"/>
       <c r="K20" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L20" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3367,30 +3638,30 @@
         <v>18</v>
       </c>
       <c r="C21" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="E21" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="F21" s="19" t="s">
         <v>127</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>129</v>
       </c>
       <c r="G21" s="14"/>
       <c r="H21" s="15">
         <v>43342</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J21" s="17"/>
       <c r="K21" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3400,7 +3671,7 @@
       <c r="C22" s="19"/>
       <c r="D22" s="19"/>
       <c r="E22" s="19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F22" s="19"/>
       <c r="G22" s="14"/>
@@ -3408,14 +3679,14 @@
         <v>43342</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J22" s="17"/>
       <c r="K22" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L22" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3425,7 +3696,7 @@
       <c r="C23" s="19"/>
       <c r="D23" s="19"/>
       <c r="E23" s="19" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F23" s="19"/>
       <c r="G23" s="14"/>
@@ -3433,14 +3704,14 @@
         <v>43342</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J23" s="17"/>
       <c r="K23" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L23" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3449,10 +3720,10 @@
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="19" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F24" s="19"/>
       <c r="G24" s="14"/>
@@ -3460,14 +3731,14 @@
         <v>43345</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J24" s="17"/>
       <c r="K24" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3480,41 +3751,41 @@
         <v>43347</v>
       </c>
       <c r="I25" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J25" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="L25" s="17" t="s">
         <v>133</v>
-      </c>
-      <c r="J25" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="K25" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="L25" s="17" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="26" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
       <c r="B26" s="18"/>
       <c r="C26" s="19"/>
       <c r="D26" s="19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E26" s="19"/>
       <c r="F26" s="19" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G26" s="14"/>
       <c r="H26" s="15">
         <v>43345</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J26" s="17"/>
       <c r="K26" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L26" s="17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="2:12" s="1" customFormat="1" ht="20.149999999999999" customHeight="1">
@@ -3523,21 +3794,21 @@
       <c r="D27" s="19"/>
       <c r="E27" s="19"/>
       <c r="F27" s="19" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G27" s="14"/>
       <c r="H27" s="15">
         <v>43347</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J27" s="17"/>
       <c r="K27" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="L27" s="17" t="s">
         <v>133</v>
-      </c>
-      <c r="L27" s="17" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="28" spans="2:12" ht="20.149999999999999" customHeight="1">
@@ -3551,16 +3822,16 @@
         <v>43346</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J28" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="L28" s="17" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="2:12" ht="20.149999999999999" customHeight="1">
@@ -3569,14 +3840,14 @@
         <v>43346</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J29" s="17"/>
       <c r="K29" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L29" s="17" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="2:12">
@@ -3585,14 +3856,14 @@
         <v>43357</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J30" s="24" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K30" s="17"/>
       <c r="L30" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="2:12">
@@ -3600,11 +3871,11 @@
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
       <c r="J31" s="24" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K31" s="17"/>
       <c r="L31" s="17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="2:12">
@@ -4052,7 +4323,7 @@
       <c r="B179" s="23"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="0.98" bottom="0.98" header="0.51" footer="0.51"/>
   <pageSetup paperSize="9" orientation="landscape"/>
 </worksheet>

</xml_diff>